<commit_message>
Maj règle de gestion 6234993b262dad5b444318eeefd97143e26d5dfa
</commit_message>
<xml_diff>
--- a/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
+++ b/450-contenu-fhir---ajout-des-objets-demandeorientation-decision-droitprestation/ig/CodeSystem-tddui-basic-decision-identifier.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="52">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-19T09:35:09+00:00</t>
+    <t>2026-06-08T15:24:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -123,7 +123,7 @@
     <t>Count</t>
   </si>
   <si>
-    <t>4</t>
+    <t>5</t>
   </si>
   <si>
     <t>Level</t>
@@ -145,6 +145,12 @@
   </si>
   <si>
     <t>Identifiant principal de la décision</t>
+  </si>
+  <si>
+    <t>IDDECISIONMAJ</t>
+  </si>
+  <si>
+    <t>Identifiant révisé de la décision</t>
   </si>
   <si>
     <t>NUMENREG</t>
@@ -472,7 +478,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -537,6 +543,18 @@
       </c>
       <c r="D5" s="2"/>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="2">
+        <v>41</v>
+      </c>
+      <c r="B6" t="s" s="2">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s" s="2">
+        <v>51</v>
+      </c>
+      <c r="D6" s="2"/>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>